<commit_message>
feat(outreach): lock launch offer — 2000 DH vitrine, live in 2-3 days, free SEO+GBP
Concrete offer folded into all 22 non-riad lead messages + workbook + playbook;
riads keep custom booking-site launch pricing. Speed (2-3 days) featured as the
lead hook. Regenerated wereact-leads.xlsx + leads-batch-01.md.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/outreach/wereact-leads.xlsx
+++ b/docs/outreach/wereact-leads.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Casa De Marrakech cumule plus de 750 avis sur Booking — bravo ! Mais chaque réservation vous coûte 15 à 25 % de commission, et nous n'avons trouvé aucun site de réservation directe à votre nom. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Casa De Marrakech cumule plus de 750 avis sur Booking — bravo ! Mais chaque réservation vous coûte 15 à 25 % de commission, et nous n'avons trouvé aucun site de réservation directe à votre nom. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Le Riad Beni Sidel a déjà 398 excellents avis sur Booking sans jamais avoir eu de site à lui — chaque nuit vendue profite d'abord à la plateforme. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Le Riad Beni Sidel a déjà 398 excellents avis sur Booking sans jamais avoir eu de site à lui — chaque nuit vendue profite d'abord à la plateforme. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Avec un 9,6 sur Booking et une jolie page Instagram, il ne manque au Riad Al Wifak qu'un site à lui pour transformer ces abonnés en réservations directes, sans commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Avec un 9,6 sur Booking et une jolie page Instagram, il ne manque au Riad Al Wifak qu'un site à lui pour transformer ces abonnés en réservations directes, sans commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Le Riad Jnan El Cadi affiche 9,3/10 sur Booking et une belle page Instagram, mais reste invisible sur Google en dehors des plateformes qui prennent leur commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Le Riad Jnan El Cadi affiche 9,3/10 sur Booking et une belle page Instagram, mais reste invisible sur Google en dehors des plateformes qui prennent leur commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Le Riad Laichi a de bons avis et un compte Instagram, mais aucun site perso pour convertir ces abonnés en réservations sans commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Le Riad Laichi a de bons avis et un compte Instagram, mais aucun site perso pour convertir ces abonnés en réservations sans commission. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 À deux pas de Jemaa el-Fna, le Riad Atlas Guest House a de bons avis mais aucun site à lui pour réserver en direct — donc 15 à 25 % de commission sur chaque nuit. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 À deux pas de Jemaa el-Fna, le Riad Atlas Guest House a de bons avis mais aucun site à lui pour réserver en direct — donc 15 à 25 % de commission sur chaque nuit. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Le Riad La Calèche a sa piscine, ses avis, sa page Facebook — il ne manque que le site pour arrêter de reverser 15 à 25 % à chaque réservation. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques établissements ce mois-ci. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Le Riad La Calèche a sa piscine, ses avis, sa page Facebook — il ne manque que le site pour arrêter de reverser 15 à 25 % à chaque réservation. Chez WeReact — studio web à Marrakech — nous créons des sites de réservation directe pour riads (exemple : kasbahangour.com). 🎉 Offre de lancement : tarif préférentiel + fondations SEO et fiche Google Business OFFERTES, avec une première version en ligne en quelques jours. On en parle 10 minutes cette semaine ? — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Toute la rue Ibn Aïcha connaît vos grillades, mais un client qui vous cherche sur Google ce soir ne trouve qu'un avis TripAdvisor. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Toute la rue Ibn Aïcha connaît vos grillades, mais un client qui vous cherche sur Google ce soir ne trouve qu'un avis TripAdvisor. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Même votre ancien nom de domaine chezouazzani.com a disparu du web — un site d'une page avec la carte (tanjia !) et un accès WhatsApp direct vous remettrait devant les touristes. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Même votre ancien nom de domaine chezouazzani.com a disparu du web — un site d'une page avec la carte (tanjia !) et un accès WhatsApp direct vous remettrait devant les touristes. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Institution de l'avenue Mohammed V, Café Elite mérite mieux qu'un lien mort vers un portail générique quand on tape son nom sur Google. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Institution de l'avenue Mohammed V, Café Elite mérite mieux qu'un lien mort vers un portail générique quand on tape son nom sur Google. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Avec 4,6 étoiles et un menu à moins de 7 € juste à côté de Jamaa El Fna, Gargot est une pépite que les voyageurs ne trouvent qu'en tombant par hasard sur TripAdvisor. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Avec 4,6 étoiles et un menu à moins de 7 € juste à côté de Jamaa El Fna, Gargot est une pépite que les voyageurs ne trouvent qu'en tombant par hasard sur TripAdvisor. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos habitués vous adorent rue Bani Marine, mais sur Google votre nom ne renvoie qu'à des pages Facebook non réclamées et des annuaires poussiéreux. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos habitués vous adorent rue Bani Marine, mais sur Google votre nom ne renvoie qu'à des pages Facebook non réclamées et des annuaires poussiéreux. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos glaces aux saveurs marocaines font le buzz sur Instagram, mais aucune page ne raconte votre histoire aux touristes de passage rue Mouassine. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos glaces aux saveurs marocaines font le buzz sur Instagram, mais aucune page ne raconte votre histoire aux touristes de passage rue Mouassine. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre vue sur l'Atlas est notée 4,7/5, mais les visiteurs qui cherchent « rooftop médina réservation » ne tombent que sur TripAdvisor et Instagram. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre vue sur l'Atlas est notée 4,7/5, mais les visiteurs qui cherchent « rooftop médina réservation » ne tombent que sur TripAdvisor et Instagram. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Face au Palais des Congrès, votre terrasse est un repère des habitués — mais aucun site ne présente votre carte aux touristes des hôtels du quartier. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Face au Palais des Congrès, votre terrasse est un repère des habitués — mais aucun site ne présente votre carte aux touristes des hôtels du quartier. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Avec 18 000 abonnées mais zéro lien de réservation en bio, chaque cliente doit écrire en DM pour un rendez-vous. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Avec 18 000 abonnées mais zéro lien de réservation en bio, chaque cliente doit écrire en DM pour un rendez-vous. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre domaine beautylab.ma affiche une erreur alors que votre salon tourne à plein avec 21 000 abonnées — un vrai site actif évite de perdre les clientes qui tombent sur cette page en erreur. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre domaine beautylab.ma affiche une erreur alors que votre salon tourne à plein avec 21 000 abonnées — un vrai site actif évite de perdre les clientes qui tombent sur cette page en erreur. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos 9 300 abonnées ne trouvent aucun site ni fiche à votre nom — vous passez à côté des recherches « institut beauté Guéliz ». Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos 9 300 abonnées ne trouvent aucun site ni fiche à votre nom — vous passez à côté des recherches « institut beauté Guéliz ». Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos tresses et box braids cartonnent en Reels — un site vitrine avec galerie et prise de rendez-vous capterait les clientes qui tapent « salon coiffure afro Marrakech » sur Google. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos tresses et box braids cartonnent en Reels — un site vitrine avec galerie et prise de rendez-vous capterait les clientes qui tapent « salon coiffure afro Marrakech » sur Google. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre adresse email en @le7emesens.ma prouve que vous aviez pensé à un site, mais le domaine ne pointe vers aucune page aujourd'hui. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre adresse email en @le7emesens.ma prouve que vous aviez pensé à un site, mais le domaine ne pointe vers aucune page aujourd'hui. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre ancien site funfitness.ma ne répond plus, alors que des concurrents trônent en tête de Google — le moment idéal pour relancer une vraie vitrine. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre ancien site funfitness.ma ne répond plus, alors que des concurrents trônent en tête de Google — le moment idéal pour relancer une vraie vitrine. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos clientes vous trouvent sur Instagram mais doivent deviner vos tarifs en DM — un site avec grille tarifaire et réservation transformerait vos abonnés en rendez-vous confirmés. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos clientes vous trouvent sur Instagram mais doivent deviner vos tarifs en DM — un site avec grille tarifaire et réservation transformerait vos abonnés en rendez-vous confirmés. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre fiche Google a disparu (page 404), il ne reste qu'Instagram pour exister en ligne — un vrai site vous protège de dépendre entièrement des algorithmes. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre fiche Google a disparu (page 404), il ne reste qu'Instagram pour exister en ligne — un vrai site vous protège de dépendre entièrement des algorithmes. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre atelier est noté en or sur TripAdvisor, mais votre site déclenche une alerte de sécurité avant même que vos visiteurs voient vos tajines — combien abandonnent sur cet écran rouge ? Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre atelier est noté en or sur TripAdvisor, mais votre site déclenche une alerte de sécurité avant même que vos visiteurs voient vos tajines — combien abandonnent sur cet écran rouge ? Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre site deniztours.com ne se charge plus (erreur serveur), alors qu'un client qui compare les agences à l'aéroport a besoin de voir vos tarifs tout de suite. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre site deniztours.com ne se charge plus (erreur serveur), alors qu'un client qui compare les agences à l'aéroport a besoin de voir vos tarifs tout de suite. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Vos clients vous découvrent entre deux stories Instagram, mais un traiteur haut de gamme sans page de réservation perd chaque semaine des demandes de devis. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Vos clients vous découvrent entre deux stories Instagram, mais un traiteur haut de gamme sans page de réservation perd chaque semaine des demandes de devis. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Votre poterie mérite une vitrine capable de vendre à l'international, pas seulement une page Facebook que les touristes oublient une fois rentrés. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Votre poterie mérite une vitrine capable de vendre à l'international, pas seulement une page Facebook que les touristes oublient une fois rentrés. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Autour du lac Lalla Takerkoust, vos concurrents captent la réservation avant même l'arrivée du client via leur site — vous comptez encore sur Facebook pour être trouvé. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Autour du lac Lalla Takerkoust, vos concurrents captent la réservation avant même l'arrivée du client via leur site — vous comptez encore sur Facebook pour être trouvé. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Bonjour 👋 Un randonneur qui prépare son ascension du Toubkal trois mois à l'avance depuis l'étranger a besoin d'un site pour vous trouver et réserver — pas seulement d'un profil Facebook. Chez WeReact — studio web à Marrakech — nous créons des sites rapides, bilingues et pensés pour ramener des clients. 🎉 Pour le lancement de notre studio, nous offrons un tarif de lancement + les fondations SEO offertes à quelques entreprises de Marrakech ce mois-ci. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
+          <t>Bonjour 👋 Un randonneur qui prépare son ascension du Toubkal trois mois à l'avance depuis l'étranger a besoin d'un site pour vous trouver et réserver — pas seulement d'un profil Facebook. Chez WeReact — studio web à Marrakech — nous créons des sites rapides et bilingues qui ramènent des clients. 🎉 Offre de lancement : votre site vitrine professionnel à 2000 DH, en ligne en 2 à 3 jours, avec les fondations SEO + votre fiche Google Business optimisée OFFERTES. On en discute 10 minutes cette semaine ? Nos réalisations : wereact.agency/fr/work — L'équipe WeReact, +212 602-258009</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2351,7 +2351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2429,28 +2429,28 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>OFFRE DE LANCEMENT WeReact (à personnaliser)</t>
+          <t>OFFRE DE LANCEMENT WeReact</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>• Réservée aux 5 premières entreprises de Marrakech qui démarrent ce mois-ci (rareté vraie = crédible).</t>
+          <t>• Site vitrine professionnel : 2000 DH (prix de lancement), EN LIGNE EN 2 À 3 JOURS.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>• Tarif de lancement réduit (recommandé : −20 à −30% OU un prix de lancement affiché, ex. site vitrine à partir de 3 500 MAD).</t>
+          <t>• OFFERT avec chaque site : fondations SEO + fiche Google Business optimisée.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>• OFFERT : fondations SEO + fiche Google Business optimisée (valeur ~1 500 MAD).</t>
+          <t>• Réservé aux 5 premières entreprises de Marrakech qui démarrent ce mois-ci (rareté vraie = crédible).</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,21 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>• Riads / sites de réservation : projet sur mesure au tarif de lancement, avec les mêmes bonus SEO + Google Business offerts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>• Pourquoi limité : « parce que nous lançons notre studio et voulons quelques belles références locales. » (vrai + donne envie d'en être).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>• Argument massue : rapide (2-3 jours), pas cher (2000 DH), et sans risque (SEO offert + tarif de lancement). Peu d'excuses pour dire non.</t>
         </is>
       </c>
     </row>

</xml_diff>